<commit_message>
Workshop 2 exercise 1 finished
</commit_message>
<xml_diff>
--- a/data/titanic-clean.xlsx
+++ b/data/titanic-clean.xlsx
@@ -690,7 +690,7 @@
         </is>
       </c>
       <c r="F7" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -1170,7 +1170,7 @@
         </is>
       </c>
       <c r="F19" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -1248,7 +1248,7 @@
         </is>
       </c>
       <c r="F21" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -1529,7 +1529,7 @@
         </is>
       </c>
       <c r="F28" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G28" t="inlineStr">
         <is>
@@ -1611,7 +1611,7 @@
         </is>
       </c>
       <c r="F30" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G30" t="inlineStr">
         <is>
@@ -1650,7 +1650,7 @@
         </is>
       </c>
       <c r="F31" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G31" t="inlineStr">
         <is>
@@ -1728,7 +1728,7 @@
         </is>
       </c>
       <c r="F33" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G33" t="inlineStr">
         <is>
@@ -1771,7 +1771,7 @@
         </is>
       </c>
       <c r="F34" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G34" t="inlineStr">
         <is>
@@ -1927,7 +1927,7 @@
         </is>
       </c>
       <c r="F38" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G38" t="inlineStr">
         <is>
@@ -2161,7 +2161,7 @@
         </is>
       </c>
       <c r="F44" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G44" t="inlineStr">
         <is>
@@ -2278,7 +2278,7 @@
         </is>
       </c>
       <c r="F47" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G47" t="inlineStr">
         <is>
@@ -2317,7 +2317,7 @@
         </is>
       </c>
       <c r="F48" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G48" t="inlineStr">
         <is>
@@ -2356,7 +2356,7 @@
         </is>
       </c>
       <c r="F49" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G49" t="inlineStr">
         <is>
@@ -2395,7 +2395,7 @@
         </is>
       </c>
       <c r="F50" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G50" t="inlineStr">
         <is>
@@ -2676,7 +2676,7 @@
         </is>
       </c>
       <c r="F57" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G57" t="inlineStr">
         <is>
@@ -2758,7 +2758,7 @@
         </is>
       </c>
       <c r="F59" t="n">
-        <v>28.5</v>
+        <v>28</v>
       </c>
       <c r="G59" t="inlineStr">
         <is>
@@ -3035,7 +3035,7 @@
         </is>
       </c>
       <c r="F66" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G66" t="inlineStr">
         <is>
@@ -3074,7 +3074,7 @@
         </is>
       </c>
       <c r="F67" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G67" t="inlineStr">
         <is>
@@ -3511,7 +3511,7 @@
         </is>
       </c>
       <c r="F78" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G78" t="inlineStr">
         <is>
@@ -3550,7 +3550,7 @@
         </is>
       </c>
       <c r="F79" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G79" t="inlineStr">
         <is>
@@ -3589,7 +3589,7 @@
         </is>
       </c>
       <c r="F80" t="n">
-        <v>0.83</v>
+        <v>0</v>
       </c>
       <c r="G80" t="inlineStr">
         <is>
@@ -3745,7 +3745,7 @@
         </is>
       </c>
       <c r="F84" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G84" t="inlineStr">
         <is>
@@ -3940,7 +3940,7 @@
         </is>
       </c>
       <c r="F89" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G89" t="inlineStr">
         <is>
@@ -4260,7 +4260,7 @@
         </is>
       </c>
       <c r="F97" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G97" t="inlineStr">
         <is>
@@ -4502,7 +4502,7 @@
         </is>
       </c>
       <c r="F103" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G103" t="inlineStr">
         <is>
@@ -4740,7 +4740,7 @@
         </is>
       </c>
       <c r="F109" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G109" t="inlineStr">
         <is>
@@ -4818,7 +4818,7 @@
         </is>
       </c>
       <c r="F111" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G111" t="inlineStr">
         <is>
@@ -4900,7 +4900,7 @@
         </is>
       </c>
       <c r="F113" t="n">
-        <v>14.5</v>
+        <v>14</v>
       </c>
       <c r="G113" t="inlineStr">
         <is>
@@ -5095,7 +5095,7 @@
         </is>
       </c>
       <c r="F118" t="n">
-        <v>70.5</v>
+        <v>70</v>
       </c>
       <c r="G118" t="inlineStr">
         <is>
@@ -5294,7 +5294,7 @@
         </is>
       </c>
       <c r="F123" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G123" t="inlineStr">
         <is>
@@ -5333,7 +5333,7 @@
         </is>
       </c>
       <c r="F124" t="n">
-        <v>32.5</v>
+        <v>32</v>
       </c>
       <c r="G124" t="inlineStr">
         <is>
@@ -5372,7 +5372,7 @@
         </is>
       </c>
       <c r="F125" t="n">
-        <v>32.5</v>
+        <v>32</v>
       </c>
       <c r="G125" t="inlineStr">
         <is>
@@ -5497,7 +5497,7 @@
         </is>
       </c>
       <c r="F128" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G128" t="inlineStr">
         <is>
@@ -5575,7 +5575,7 @@
         </is>
       </c>
       <c r="F130" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G130" t="inlineStr">
         <is>
@@ -6059,7 +6059,7 @@
         </is>
       </c>
       <c r="F142" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G142" t="inlineStr">
         <is>
@@ -6371,7 +6371,7 @@
         </is>
       </c>
       <c r="F150" t="n">
-        <v>36.5</v>
+        <v>36</v>
       </c>
       <c r="G150" t="inlineStr">
         <is>
@@ -6535,7 +6535,7 @@
         </is>
       </c>
       <c r="F154" t="n">
-        <v>55.5</v>
+        <v>55</v>
       </c>
       <c r="G154" t="inlineStr">
         <is>
@@ -6574,7 +6574,7 @@
         </is>
       </c>
       <c r="F155" t="n">
-        <v>40.5</v>
+        <v>40</v>
       </c>
       <c r="G155" t="inlineStr">
         <is>
@@ -6613,7 +6613,7 @@
         </is>
       </c>
       <c r="F156" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G156" t="inlineStr">
         <is>
@@ -6769,7 +6769,7 @@
         </is>
       </c>
       <c r="F160" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G160" t="inlineStr">
         <is>
@@ -6808,7 +6808,7 @@
         </is>
       </c>
       <c r="F161" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G161" t="inlineStr">
         <is>
@@ -7081,7 +7081,7 @@
         </is>
       </c>
       <c r="F168" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G168" t="inlineStr">
         <is>
@@ -7163,7 +7163,7 @@
         </is>
       </c>
       <c r="F170" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G170" t="inlineStr">
         <is>
@@ -7483,7 +7483,7 @@
         </is>
       </c>
       <c r="F178" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G178" t="inlineStr">
         <is>
@@ -7643,7 +7643,7 @@
         </is>
       </c>
       <c r="F182" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G182" t="inlineStr">
         <is>
@@ -7682,7 +7682,7 @@
         </is>
       </c>
       <c r="F183" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G183" t="inlineStr">
         <is>
@@ -7842,7 +7842,7 @@
         </is>
       </c>
       <c r="F187" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G187" t="inlineStr">
         <is>
@@ -7885,7 +7885,7 @@
         </is>
       </c>
       <c r="F188" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G188" t="inlineStr">
         <is>
@@ -8287,7 +8287,7 @@
         </is>
       </c>
       <c r="F198" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G198" t="inlineStr">
         <is>
@@ -8365,7 +8365,7 @@
         </is>
       </c>
       <c r="F200" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G200" t="inlineStr">
         <is>
@@ -8482,7 +8482,7 @@
         </is>
       </c>
       <c r="F203" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G203" t="inlineStr">
         <is>
@@ -8560,7 +8560,7 @@
         </is>
       </c>
       <c r="F205" t="n">
-        <v>45.5</v>
+        <v>45</v>
       </c>
       <c r="G205" t="inlineStr">
         <is>
@@ -8997,7 +8997,7 @@
         </is>
       </c>
       <c r="F216" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G216" t="inlineStr">
         <is>
@@ -9356,7 +9356,7 @@
         </is>
       </c>
       <c r="F225" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G225" t="inlineStr">
         <is>
@@ -9516,7 +9516,7 @@
         </is>
       </c>
       <c r="F229" t="n">
-        <v>20.5</v>
+        <v>20</v>
       </c>
       <c r="G229" t="inlineStr">
         <is>
@@ -9594,7 +9594,7 @@
         </is>
       </c>
       <c r="F231" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G231" t="inlineStr">
         <is>
@@ -9832,7 +9832,7 @@
         </is>
       </c>
       <c r="F237" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G237" t="inlineStr">
         <is>
@@ -10027,7 +10027,7 @@
         </is>
       </c>
       <c r="F242" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G242" t="inlineStr">
         <is>
@@ -10066,7 +10066,7 @@
         </is>
       </c>
       <c r="F243" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G243" t="inlineStr">
         <is>
@@ -10425,7 +10425,7 @@
         </is>
       </c>
       <c r="F252" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G252" t="inlineStr">
         <is>
@@ -10667,7 +10667,7 @@
         </is>
       </c>
       <c r="F258" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G258" t="inlineStr">
         <is>
@@ -10827,7 +10827,7 @@
         </is>
       </c>
       <c r="F262" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G262" t="inlineStr">
         <is>
@@ -10991,7 +10991,7 @@
         </is>
       </c>
       <c r="F266" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G266" t="inlineStr">
         <is>
@@ -11233,7 +11233,7 @@
         </is>
       </c>
       <c r="F272" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G272" t="inlineStr">
         <is>
@@ -11393,7 +11393,7 @@
         </is>
       </c>
       <c r="F276" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G276" t="inlineStr">
         <is>
@@ -11514,7 +11514,7 @@
         </is>
       </c>
       <c r="F279" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G279" t="inlineStr">
         <is>
@@ -11787,7 +11787,7 @@
         </is>
       </c>
       <c r="F286" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G286" t="inlineStr">
         <is>
@@ -12228,7 +12228,7 @@
         </is>
       </c>
       <c r="F297" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G297" t="inlineStr">
         <is>
@@ -12267,7 +12267,7 @@
         </is>
       </c>
       <c r="F298" t="n">
-        <v>23.5</v>
+        <v>23</v>
       </c>
       <c r="G298" t="inlineStr">
         <is>
@@ -12349,7 +12349,7 @@
         </is>
       </c>
       <c r="F300" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G300" t="inlineStr">
         <is>
@@ -12435,7 +12435,7 @@
         </is>
       </c>
       <c r="F302" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G302" t="inlineStr">
         <is>
@@ -12474,7 +12474,7 @@
         </is>
       </c>
       <c r="F303" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G303" t="inlineStr">
         <is>
@@ -12552,7 +12552,7 @@
         </is>
       </c>
       <c r="F305" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G305" t="inlineStr">
         <is>
@@ -12595,7 +12595,7 @@
         </is>
       </c>
       <c r="F306" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G306" t="inlineStr">
         <is>
@@ -12634,7 +12634,7 @@
         </is>
       </c>
       <c r="F307" t="n">
-        <v>0.92</v>
+        <v>0</v>
       </c>
       <c r="G307" t="inlineStr">
         <is>
@@ -12677,7 +12677,7 @@
         </is>
       </c>
       <c r="F308" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G308" t="inlineStr">
         <is>
@@ -13403,7 +13403,7 @@
         </is>
       </c>
       <c r="F326" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G326" t="inlineStr">
         <is>
@@ -13649,7 +13649,7 @@
         </is>
       </c>
       <c r="F332" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G332" t="inlineStr">
         <is>
@@ -13688,7 +13688,7 @@
         </is>
       </c>
       <c r="F333" t="n">
-        <v>45.5</v>
+        <v>45</v>
       </c>
       <c r="G333" t="inlineStr">
         <is>
@@ -13813,7 +13813,7 @@
         </is>
       </c>
       <c r="F336" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G336" t="inlineStr">
         <is>
@@ -13852,7 +13852,7 @@
         </is>
       </c>
       <c r="F337" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G337" t="inlineStr">
         <is>
@@ -14344,7 +14344,7 @@
         </is>
       </c>
       <c r="F349" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G349" t="inlineStr">
         <is>
@@ -14500,7 +14500,7 @@
         </is>
       </c>
       <c r="F353" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G353" t="inlineStr">
         <is>
@@ -14621,7 +14621,7 @@
         </is>
       </c>
       <c r="F356" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G356" t="inlineStr">
         <is>
@@ -14781,7 +14781,7 @@
         </is>
       </c>
       <c r="F360" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G360" t="inlineStr">
         <is>
@@ -14820,7 +14820,7 @@
         </is>
       </c>
       <c r="F361" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G361" t="inlineStr">
         <is>
@@ -15015,7 +15015,7 @@
         </is>
       </c>
       <c r="F366" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G366" t="inlineStr">
         <is>
@@ -15136,7 +15136,7 @@
         </is>
       </c>
       <c r="F369" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G369" t="inlineStr">
         <is>
@@ -15175,7 +15175,7 @@
         </is>
       </c>
       <c r="F370" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G370" t="inlineStr">
         <is>
@@ -15456,7 +15456,7 @@
         </is>
       </c>
       <c r="F377" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G377" t="inlineStr">
         <is>
@@ -15811,7 +15811,7 @@
         </is>
       </c>
       <c r="F386" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G386" t="inlineStr">
         <is>
@@ -15967,7 +15967,7 @@
         </is>
       </c>
       <c r="F390" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G390" t="inlineStr">
         <is>
@@ -16798,7 +16798,7 @@
         </is>
       </c>
       <c r="F411" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G411" t="inlineStr">
         <is>
@@ -16837,7 +16837,7 @@
         </is>
       </c>
       <c r="F412" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G412" t="inlineStr">
         <is>
@@ -16876,7 +16876,7 @@
         </is>
       </c>
       <c r="F413" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G413" t="inlineStr">
         <is>
@@ -16958,7 +16958,7 @@
         </is>
       </c>
       <c r="F415" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G415" t="inlineStr">
         <is>
@@ -17036,7 +17036,7 @@
         </is>
       </c>
       <c r="F417" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G417" t="inlineStr">
         <is>
@@ -17231,7 +17231,7 @@
         </is>
       </c>
       <c r="F422" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G422" t="inlineStr">
         <is>
@@ -17426,7 +17426,7 @@
         </is>
       </c>
       <c r="F427" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G427" t="inlineStr">
         <is>
@@ -17543,7 +17543,7 @@
         </is>
       </c>
       <c r="F430" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G430" t="inlineStr">
         <is>
@@ -17668,7 +17668,7 @@
         </is>
       </c>
       <c r="F433" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G433" t="inlineStr">
         <is>
@@ -18187,7 +18187,7 @@
         </is>
       </c>
       <c r="F446" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G446" t="inlineStr">
         <is>
@@ -18468,7 +18468,7 @@
         </is>
       </c>
       <c r="F453" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G453" t="inlineStr">
         <is>
@@ -18593,7 +18593,7 @@
         </is>
       </c>
       <c r="F456" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G456" t="inlineStr">
         <is>
@@ -18714,7 +18714,7 @@
         </is>
       </c>
       <c r="F459" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G459" t="inlineStr">
         <is>
@@ -18796,7 +18796,7 @@
         </is>
       </c>
       <c r="F461" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G461" t="inlineStr">
         <is>
@@ -18999,7 +18999,7 @@
         </is>
       </c>
       <c r="F466" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G466" t="inlineStr">
         <is>
@@ -19077,7 +19077,7 @@
         </is>
       </c>
       <c r="F468" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G468" t="inlineStr">
         <is>
@@ -19155,7 +19155,7 @@
         </is>
       </c>
       <c r="F470" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G470" t="inlineStr">
         <is>
@@ -19194,7 +19194,7 @@
         </is>
       </c>
       <c r="F471" t="n">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="G471" t="inlineStr">
         <is>
@@ -19233,7 +19233,7 @@
         </is>
       </c>
       <c r="F472" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G472" t="inlineStr">
         <is>
@@ -19432,7 +19432,7 @@
         </is>
       </c>
       <c r="F477" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G477" t="inlineStr">
         <is>
@@ -19670,7 +19670,7 @@
         </is>
       </c>
       <c r="F483" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G483" t="inlineStr">
         <is>
@@ -19830,7 +19830,7 @@
         </is>
       </c>
       <c r="F487" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G487" t="inlineStr">
         <is>
@@ -20033,7 +20033,7 @@
         </is>
       </c>
       <c r="F492" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G492" t="inlineStr">
         <is>
@@ -20232,7 +20232,7 @@
         </is>
       </c>
       <c r="F497" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G497" t="inlineStr">
         <is>
@@ -20314,7 +20314,7 @@
         </is>
       </c>
       <c r="F499" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G499" t="inlineStr">
         <is>
@@ -20513,7 +20513,7 @@
         </is>
       </c>
       <c r="F504" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G504" t="inlineStr">
         <is>
@@ -20716,7 +20716,7 @@
         </is>
       </c>
       <c r="F509" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G509" t="inlineStr">
         <is>
@@ -20872,7 +20872,7 @@
         </is>
       </c>
       <c r="F513" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G513" t="inlineStr">
         <is>
@@ -21118,7 +21118,7 @@
         </is>
       </c>
       <c r="F519" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G519" t="inlineStr">
         <is>
@@ -21317,7 +21317,7 @@
         </is>
       </c>
       <c r="F524" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G524" t="inlineStr">
         <is>
@@ -21399,7 +21399,7 @@
         </is>
       </c>
       <c r="F526" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G526" t="inlineStr">
         <is>
@@ -21438,7 +21438,7 @@
         </is>
       </c>
       <c r="F527" t="n">
-        <v>40.5</v>
+        <v>40</v>
       </c>
       <c r="G527" t="inlineStr">
         <is>
@@ -21516,7 +21516,7 @@
         </is>
       </c>
       <c r="F529" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G529" t="inlineStr">
         <is>
@@ -21676,7 +21676,7 @@
         </is>
       </c>
       <c r="F533" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G533" t="inlineStr">
         <is>
@@ -21754,7 +21754,7 @@
         </is>
       </c>
       <c r="F535" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G535" t="inlineStr">
         <is>
@@ -21953,7 +21953,7 @@
         </is>
       </c>
       <c r="F540" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G540" t="inlineStr">
         <is>
@@ -22316,7 +22316,7 @@
         </is>
       </c>
       <c r="F549" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G549" t="inlineStr">
         <is>
@@ -22515,7 +22515,7 @@
         </is>
       </c>
       <c r="F554" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G554" t="inlineStr">
         <is>
@@ -22714,7 +22714,7 @@
         </is>
       </c>
       <c r="F559" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G559" t="inlineStr">
         <is>
@@ -22835,7 +22835,7 @@
         </is>
       </c>
       <c r="F562" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G562" t="inlineStr">
         <is>
@@ -22952,7 +22952,7 @@
         </is>
       </c>
       <c r="F565" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G565" t="inlineStr">
         <is>
@@ -22991,7 +22991,7 @@
         </is>
       </c>
       <c r="F566" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G566" t="inlineStr">
         <is>
@@ -23147,7 +23147,7 @@
         </is>
       </c>
       <c r="F570" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G570" t="inlineStr">
         <is>
@@ -23350,7 +23350,7 @@
         </is>
       </c>
       <c r="F575" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G575" t="inlineStr">
         <is>
@@ -23549,7 +23549,7 @@
         </is>
       </c>
       <c r="F580" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G580" t="inlineStr">
         <is>
@@ -23791,7 +23791,7 @@
         </is>
       </c>
       <c r="F586" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G586" t="inlineStr">
         <is>
@@ -23994,7 +23994,7 @@
         </is>
       </c>
       <c r="F591" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G591" t="inlineStr">
         <is>
@@ -24154,7 +24154,7 @@
         </is>
       </c>
       <c r="F595" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G595" t="inlineStr">
         <is>
@@ -24271,7 +24271,7 @@
         </is>
       </c>
       <c r="F598" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G598" t="inlineStr">
         <is>
@@ -24349,7 +24349,7 @@
         </is>
       </c>
       <c r="F600" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G600" t="inlineStr">
         <is>
@@ -24470,7 +24470,7 @@
         </is>
       </c>
       <c r="F603" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G603" t="inlineStr">
         <is>
@@ -24509,7 +24509,7 @@
         </is>
       </c>
       <c r="F604" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G604" t="inlineStr">
         <is>
@@ -24864,7 +24864,7 @@
         </is>
       </c>
       <c r="F613" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G613" t="inlineStr">
         <is>
@@ -24903,7 +24903,7 @@
         </is>
       </c>
       <c r="F614" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G614" t="inlineStr">
         <is>
@@ -24942,7 +24942,7 @@
         </is>
       </c>
       <c r="F615" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G615" t="inlineStr">
         <is>
@@ -25582,7 +25582,7 @@
         </is>
       </c>
       <c r="F631" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G631" t="inlineStr">
         <is>
@@ -25746,7 +25746,7 @@
         </is>
       </c>
       <c r="F635" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G635" t="inlineStr">
         <is>
@@ -25980,7 +25980,7 @@
         </is>
       </c>
       <c r="F641" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G641" t="inlineStr">
         <is>
@@ -26140,7 +26140,7 @@
         </is>
       </c>
       <c r="F645" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G645" t="inlineStr">
         <is>
@@ -26179,7 +26179,7 @@
         </is>
       </c>
       <c r="F646" t="n">
-        <v>0.75</v>
+        <v>0</v>
       </c>
       <c r="G646" t="inlineStr">
         <is>
@@ -26343,7 +26343,7 @@
         </is>
       </c>
       <c r="F650" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G650" t="inlineStr">
         <is>
@@ -26421,7 +26421,7 @@
         </is>
       </c>
       <c r="F652" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G652" t="inlineStr">
         <is>
@@ -26538,7 +26538,7 @@
         </is>
       </c>
       <c r="F655" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G655" t="inlineStr">
         <is>
@@ -26655,7 +26655,7 @@
         </is>
       </c>
       <c r="F658" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G658" t="inlineStr">
         <is>
@@ -27092,7 +27092,7 @@
         </is>
       </c>
       <c r="F669" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G669" t="inlineStr">
         <is>
@@ -27170,7 +27170,7 @@
         </is>
       </c>
       <c r="F671" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G671" t="inlineStr">
         <is>
@@ -27373,7 +27373,7 @@
         </is>
       </c>
       <c r="F676" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G676" t="inlineStr">
         <is>
@@ -27451,7 +27451,7 @@
         </is>
       </c>
       <c r="F678" t="n">
-        <v>24.5</v>
+        <v>24</v>
       </c>
       <c r="G678" t="inlineStr">
         <is>
@@ -27611,7 +27611,7 @@
         </is>
       </c>
       <c r="F682" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G682" t="inlineStr">
         <is>
@@ -28091,7 +28091,7 @@
         </is>
       </c>
       <c r="F694" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G694" t="inlineStr">
         <is>
@@ -28286,7 +28286,7 @@
         </is>
       </c>
       <c r="F699" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G699" t="inlineStr">
         <is>
@@ -28774,7 +28774,7 @@
         </is>
       </c>
       <c r="F711" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G711" t="inlineStr">
         <is>
@@ -28856,7 +28856,7 @@
         </is>
       </c>
       <c r="F713" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G713" t="inlineStr">
         <is>
@@ -29149,7 +29149,7 @@
         </is>
       </c>
       <c r="F720" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G720" t="inlineStr">
         <is>
@@ -29504,7 +29504,7 @@
         </is>
       </c>
       <c r="F729" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G729" t="inlineStr">
         <is>
@@ -29703,7 +29703,7 @@
         </is>
       </c>
       <c r="F734" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G734" t="inlineStr">
         <is>
@@ -29820,7 +29820,7 @@
         </is>
       </c>
       <c r="F737" t="n">
-        <v>28.5</v>
+        <v>28</v>
       </c>
       <c r="G737" t="inlineStr">
         <is>
@@ -29941,7 +29941,7 @@
         </is>
       </c>
       <c r="F740" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G740" t="inlineStr">
         <is>
@@ -29980,7 +29980,7 @@
         </is>
       </c>
       <c r="F741" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G741" t="inlineStr">
         <is>
@@ -30019,7 +30019,7 @@
         </is>
       </c>
       <c r="F742" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G742" t="inlineStr">
         <is>
@@ -30628,7 +30628,7 @@
         </is>
       </c>
       <c r="F757" t="n">
-        <v>0.67</v>
+        <v>0</v>
       </c>
       <c r="G757" t="inlineStr">
         <is>
@@ -30827,7 +30827,7 @@
         </is>
       </c>
       <c r="F762" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G762" t="inlineStr">
         <is>
@@ -31069,7 +31069,7 @@
         </is>
       </c>
       <c r="F768" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G768" t="inlineStr">
         <is>
@@ -31108,7 +31108,7 @@
         </is>
       </c>
       <c r="F769" t="n">
-        <v>30.5</v>
+        <v>30</v>
       </c>
       <c r="G769" t="inlineStr">
         <is>
@@ -31147,7 +31147,7 @@
         </is>
       </c>
       <c r="F770" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G770" t="inlineStr">
         <is>
@@ -31346,7 +31346,7 @@
         </is>
       </c>
       <c r="F775" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G775" t="inlineStr">
         <is>
@@ -31463,7 +31463,7 @@
         </is>
       </c>
       <c r="F778" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G778" t="inlineStr">
         <is>
@@ -31545,7 +31545,7 @@
         </is>
       </c>
       <c r="F780" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G780" t="inlineStr">
         <is>
@@ -31752,7 +31752,7 @@
         </is>
       </c>
       <c r="F785" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G785" t="inlineStr">
         <is>
@@ -32029,7 +32029,7 @@
         </is>
       </c>
       <c r="F792" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G792" t="inlineStr">
         <is>
@@ -32107,7 +32107,7 @@
         </is>
       </c>
       <c r="F794" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G794" t="inlineStr">
         <is>
@@ -32146,7 +32146,7 @@
         </is>
       </c>
       <c r="F795" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G795" t="inlineStr">
         <is>
@@ -32544,7 +32544,7 @@
         </is>
       </c>
       <c r="F805" t="n">
-        <v>0.42</v>
+        <v>0</v>
       </c>
       <c r="G805" t="inlineStr">
         <is>
@@ -32981,7 +32981,7 @@
         </is>
       </c>
       <c r="F816" t="n">
-        <v>30.5</v>
+        <v>30</v>
       </c>
       <c r="G816" t="inlineStr">
         <is>
@@ -33020,7 +33020,7 @@
         </is>
       </c>
       <c r="F817" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G817" t="inlineStr">
         <is>
@@ -33422,7 +33422,7 @@
         </is>
       </c>
       <c r="F827" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G827" t="inlineStr">
         <is>
@@ -33461,7 +33461,7 @@
         </is>
       </c>
       <c r="F828" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G828" t="inlineStr">
         <is>
@@ -33539,7 +33539,7 @@
         </is>
       </c>
       <c r="F830" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G830" t="inlineStr">
         <is>
@@ -33656,7 +33656,7 @@
         </is>
       </c>
       <c r="F833" t="n">
-        <v>0.83</v>
+        <v>0</v>
       </c>
       <c r="G833" t="inlineStr">
         <is>
@@ -33695,7 +33695,7 @@
         </is>
       </c>
       <c r="F834" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G834" t="inlineStr">
         <is>
@@ -33894,7 +33894,7 @@
         </is>
       </c>
       <c r="F839" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G839" t="inlineStr">
         <is>
@@ -33972,7 +33972,7 @@
         </is>
       </c>
       <c r="F841" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G841" t="inlineStr">
         <is>
@@ -34132,7 +34132,7 @@
         </is>
       </c>
       <c r="F845" t="n">
-        <v>34.5</v>
+        <v>34</v>
       </c>
       <c r="G845" t="inlineStr">
         <is>
@@ -34249,7 +34249,7 @@
         </is>
       </c>
       <c r="F848" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G848" t="inlineStr">
         <is>
@@ -34366,7 +34366,7 @@
         </is>
       </c>
       <c r="F851" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G851" t="inlineStr">
         <is>
@@ -34768,7 +34768,7 @@
         </is>
       </c>
       <c r="F861" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G861" t="inlineStr">
         <is>
@@ -34928,7 +34928,7 @@
         </is>
       </c>
       <c r="F865" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G865" t="inlineStr">
         <is>
@@ -35127,7 +35127,7 @@
         </is>
       </c>
       <c r="F870" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G870" t="inlineStr">
         <is>
@@ -35525,7 +35525,7 @@
         </is>
       </c>
       <c r="F880" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G880" t="inlineStr">
         <is>
@@ -35923,7 +35923,7 @@
         </is>
       </c>
       <c r="F890" t="n">
-        <v>29.69911764705882</v>
+        <v>29</v>
       </c>
       <c r="G890" t="inlineStr">
         <is>

</xml_diff>